<commit_message>
Add LeafletMap functionality; add filters + search bar
</commit_message>
<xml_diff>
--- a/src/data/InnoAtlasExampleDataSet.xlsx
+++ b/src/data/InnoAtlasExampleDataSet.xlsx
@@ -1,42 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fhvorarlberg-my.sharepoint.com/personal/woda_fhv_at/Documents/00 WORK/Innovation Atlas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\github\repos\InnoAtlas\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{7BE7C505-A5F2-6641-A718-5DD28C1F22F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F62E6A9D-9A9B-5A42-871F-DDFDD086B1F7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F3295F9-275C-4177-A4C9-59D96BD4CBF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{EF2497D2-FD32-1F43-B70B-06D4793A060E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="176">
   <si>
     <t>ID</t>
   </si>
@@ -146,130 +130,15 @@
     <t>ImageCredits</t>
   </si>
   <si>
-    <t>Customer Centricity at Gebrüder Weiß</t>
-  </si>
-  <si>
-    <t>Customer centricity for beneficial services for resilient and sustainable supply chains</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At Gebrüder Weiss, the focus is shifting to customer benefits, whereas internal processes previously dominated. Initial steps towards customer focus have been taken, such as customer journey workshops and regular customer satisfaction surveys. The aim is to better understand customer needs and develop new services and products. The surveys focus on digitalisation, resilience and sustainability. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">The project aims to strengthen customer centricity at Gebrüder Weiss in order to develop customer-oriented services and products that promote secure and sustainable supply chains. The Jobs-to-be-Done and Value Proposition Design methods are used to identify customer needs. The ‘value of pains’ method quantifies the economic benefits and environmental impact of smart services. These approaches support strategic decisions for new service solutions in the myGW customer portal, which is establishing itself as a one-stop shop for logistics services. Depending on the survey results, topics will be explored in greater depth in later project phases. </t>
-  </si>
-  <si>
-    <t>Lauterach</t>
-  </si>
-  <si>
-    <t>47.46888412739542</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9.727387439904954</t>
-  </si>
-  <si>
-    <t>https://sustainablemobilitylab.eu/praxisprojekte/autonome-logistikprozesse-bei-gebr%C3%BCder-weiss-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thomas Mazzurana </t>
-  </si>
-  <si>
-    <t>Gebrüder Weiss</t>
-  </si>
-  <si>
-    <t>April 20224</t>
-  </si>
-  <si>
-    <t>December 2024</t>
-  </si>
-  <si>
-    <t>9 months</t>
-  </si>
-  <si>
-    <t>https://www.gw-world.com/us/</t>
-  </si>
-  <si>
-    <t>ZHAW Zurich University of Applied Sciences</t>
-  </si>
-  <si>
-    <t>https://www.zhaw.ch/en/university</t>
-  </si>
-  <si>
     <t>Austria</t>
   </si>
   <si>
-    <t>Ecological</t>
-  </si>
-  <si>
-    <t>Logistics</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
     <t>Sustainable Mobility Lab</t>
   </si>
   <si>
-    <t xml:space="preserve">Commuter mobility in the 
-municipality of Satteins </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corporate mobility management in the company network </t>
-  </si>
-  <si>
-    <t xml:space="preserve">The municipality of Satteins has approximately 1,000 commuters who live in the municipality (including 270 internal commuters). The commuters' destinations are mainly the greater Feldkirch area, Vorderland, Liechtenstein and Switzerland. Satteins will become even more attractive as a place to live in the future, as a shift in commuting patterns can be expected, mainly due to new transport infrastructure. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Sustainable Mobility Lab is investigating mobility in the four-country region around Lake Constance. The municipality of Satteins is a pilot municipality in this project. The aim is to improve the mobility situation for commuters from Satteins. The focus is on working specifically with cross-border commuters. </t>
-  </si>
-  <si>
-    <t>Satteins</t>
-  </si>
-  <si>
-    <t>47.22297712637881</t>
-  </si>
-  <si>
-    <t>9.6713929109802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://sustainablemobilitylab.eu/praxisprojekte/gemeinde-satteins-pendlermobilit%C3%A4t-2 </t>
-  </si>
-  <si>
-    <t>David Madlener</t>
-  </si>
-  <si>
-    <t>ORGANISATION MISSING</t>
-  </si>
-  <si>
-    <t>January 2025</t>
-  </si>
-  <si>
-    <t>December 2025</t>
-  </si>
-  <si>
-    <t>12 months</t>
-  </si>
-  <si>
-    <t>Municipality of Satteins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.satteins.net/ </t>
-  </si>
-  <si>
-    <t>Energieinstitut Vorarlberg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.energieinstitut.at/ </t>
-  </si>
-  <si>
-    <t>e5 Team Satteins</t>
-  </si>
-  <si>
     <t>LINK MISSING</t>
   </si>
   <si>
-    <t>Anne-Marie Felder</t>
-  </si>
-  <si>
     <t>Public Transport</t>
   </si>
   <si>
@@ -310,13 +179,382 @@
   </si>
   <si>
     <t>https://www.fhv.at</t>
+  </si>
+  <si>
+    <t>Digitale Bildungsplattform Wien</t>
+  </si>
+  <si>
+    <t>E-Learning-Plattform für berufliche Weiterbildung</t>
+  </si>
+  <si>
+    <t>Vienna</t>
+  </si>
+  <si>
+    <t>https://example.at/digi-wien</t>
+  </si>
+  <si>
+    <t>TU Wien</t>
+  </si>
+  <si>
+    <t>https://tuwien.at</t>
+  </si>
+  <si>
+    <t>Wirtschaft</t>
+  </si>
+  <si>
+    <t>Bildung</t>
+  </si>
+  <si>
+    <t>Aktiv</t>
+  </si>
+  <si>
+    <t>Grüne Logistik Berlin</t>
+  </si>
+  <si>
+    <t>Nachhaltige Lieferketten in der Metropolregion</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>https://example.de/gruene-log</t>
+  </si>
+  <si>
+    <t>Fraunhofer IML</t>
+  </si>
+  <si>
+    <t>https://iml.fraunhofer.de</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Umwelt</t>
+  </si>
+  <si>
+    <t>Logistik</t>
+  </si>
+  <si>
+    <t>Soziale Integration Zürich</t>
+  </si>
+  <si>
+    <t>Integrationsprojekt für Neuzugezogene</t>
+  </si>
+  <si>
+    <t>Zurich</t>
+  </si>
+  <si>
+    <t>https://example.ch/soz-zh</t>
+  </si>
+  <si>
+    <t>ETH Zürich</t>
+  </si>
+  <si>
+    <t>https://ethz.ch</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>Soziales</t>
+  </si>
+  <si>
+    <t>Smart Mobility Paris</t>
+  </si>
+  <si>
+    <t>Intelligente Mobilitätslösungen für die Île-de-France</t>
+  </si>
+  <si>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>https://example.fr/smart-mob</t>
+  </si>
+  <si>
+    <t>SNCF</t>
+  </si>
+  <si>
+    <t>https://sncf.com</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Sonstiges</t>
+  </si>
+  <si>
+    <t>Öffentlicher Verkehr</t>
+  </si>
+  <si>
+    <t>Circular Economy Amsterdam</t>
+  </si>
+  <si>
+    <t>Kreislaufwirtschaft im Großstadtkontext</t>
+  </si>
+  <si>
+    <t>Amsterdam</t>
+  </si>
+  <si>
+    <t>https://example.nl/circular</t>
+  </si>
+  <si>
+    <t>AMS Institute</t>
+  </si>
+  <si>
+    <t>https://ams-institute.org</t>
+  </si>
+  <si>
+    <t>Netherlands</t>
+  </si>
+  <si>
+    <t>Inklusive Bildung Brüssel</t>
+  </si>
+  <si>
+    <t>Inklusive Bildungsangebote für marginalisierte Gruppen</t>
+  </si>
+  <si>
+    <t>Brussels</t>
+  </si>
+  <si>
+    <t>https://example.be/incl-edu</t>
+  </si>
+  <si>
+    <t>UCLouvain</t>
+  </si>
+  <si>
+    <t>https://uclouvain.be</t>
+  </si>
+  <si>
+    <t>Belgium</t>
+  </si>
+  <si>
+    <t>Abgeschlossen</t>
+  </si>
+  <si>
+    <t>Erneuerbare Energie Rom</t>
+  </si>
+  <si>
+    <t>Erneuerbare Energien in städtischen Gebieten</t>
+  </si>
+  <si>
+    <t>Rome</t>
+  </si>
+  <si>
+    <t>https://example.it/renew</t>
+  </si>
+  <si>
+    <t>Politecnico di Milano</t>
+  </si>
+  <si>
+    <t>https://polimi.it</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>Smart City Prag</t>
+  </si>
+  <si>
+    <t>Digitale Infrastruktur für smarte Städte</t>
+  </si>
+  <si>
+    <t>Prague</t>
+  </si>
+  <si>
+    <t>https://example.cz/smart</t>
+  </si>
+  <si>
+    <t>ČVUT Praha</t>
+  </si>
+  <si>
+    <t>https://cvut.cz</t>
+  </si>
+  <si>
+    <t>Czechia</t>
+  </si>
+  <si>
+    <t>Urbane Mobilität Warschau</t>
+  </si>
+  <si>
+    <t>Verbesserung des ÖPNV in Warschau</t>
+  </si>
+  <si>
+    <t>Warsaw</t>
+  </si>
+  <si>
+    <t>https://example.pl/urban-mob</t>
+  </si>
+  <si>
+    <t>Politechnika Warszawska</t>
+  </si>
+  <si>
+    <t>https://pw.edu.pl</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>Innovations-Hub München</t>
+  </si>
+  <si>
+    <t>Startup-Ökosystem und Technologietransfer</t>
+  </si>
+  <si>
+    <t>Munich</t>
+  </si>
+  <si>
+    <t>https://example.de/innov-muc</t>
+  </si>
+  <si>
+    <t>LMU München</t>
+  </si>
+  <si>
+    <t>https://lmu.de</t>
+  </si>
+  <si>
+    <t>Grenzlogistik Bratislava</t>
+  </si>
+  <si>
+    <t>Grenzüberschreitende Logistikkorridore</t>
+  </si>
+  <si>
+    <t>Bratislava</t>
+  </si>
+  <si>
+    <t>https://example.sk/cross-log</t>
+  </si>
+  <si>
+    <t>STU Bratislava</t>
+  </si>
+  <si>
+    <t>https://stuba.sk</t>
+  </si>
+  <si>
+    <t>Slovakia</t>
+  </si>
+  <si>
+    <t>Grüner Verkehr Ljubljana</t>
+  </si>
+  <si>
+    <t>Elektromobilität und Ladeinfrastruktur</t>
+  </si>
+  <si>
+    <t>Ljubljana</t>
+  </si>
+  <si>
+    <t>https://example.si/green-tr</t>
+  </si>
+  <si>
+    <t>Univerza v Ljubljani</t>
+  </si>
+  <si>
+    <t>https://uni-lj.si</t>
+  </si>
+  <si>
+    <t>Slovenia</t>
+  </si>
+  <si>
+    <t>Alpentourismus Innsbruck</t>
+  </si>
+  <si>
+    <t>Nachhaltiger Alpentourismus und Mobilität</t>
+  </si>
+  <si>
+    <t>Innsbruck</t>
+  </si>
+  <si>
+    <t>https://example.at/alpine</t>
+  </si>
+  <si>
+    <t>Universität Innsbruck</t>
+  </si>
+  <si>
+    <t>https://uibk.ac.at</t>
+  </si>
+  <si>
+    <t>Digitale Gesundheit Bern</t>
+  </si>
+  <si>
+    <t>Digitale Gesundheitsversorgung für ältere Menschen</t>
+  </si>
+  <si>
+    <t>Bern</t>
+  </si>
+  <si>
+    <t>https://example.ch/digi-health</t>
+  </si>
+  <si>
+    <t>Universität Bern</t>
+  </si>
+  <si>
+    <t>https://unibe.ch</t>
+  </si>
+  <si>
+    <t>Lebensmittelversorgung Lyon</t>
+  </si>
+  <si>
+    <t>Nachhaltige Lebensmittelversorgungsketten</t>
+  </si>
+  <si>
+    <t>Lyon</t>
+  </si>
+  <si>
+    <t>https://example.fr/food-supply</t>
+  </si>
+  <si>
+    <t>INRAE</t>
+  </si>
+  <si>
+    <t>https://inrae.fr</t>
+  </si>
+  <si>
+    <t>Nachhaltiger Campus Kopenhagen</t>
+  </si>
+  <si>
+    <t>Energieneutrale Hochschulcampusse</t>
+  </si>
+  <si>
+    <t>Copenhagen</t>
+  </si>
+  <si>
+    <t>https://example.dk/campus</t>
+  </si>
+  <si>
+    <t>DTU</t>
+  </si>
+  <si>
+    <t>https://dtu.dk</t>
+  </si>
+  <si>
+    <t>Denmark</t>
+  </si>
+  <si>
+    <t>Intelligentes Stromnetz Stockholm</t>
+  </si>
+  <si>
+    <t>Intelligente Stromnetze für nordische Städte</t>
+  </si>
+  <si>
+    <t>Stockholm</t>
+  </si>
+  <si>
+    <t>https://example.se/smart-grid</t>
+  </si>
+  <si>
+    <t>KTH</t>
+  </si>
+  <si>
+    <t>https://kth.se</t>
+  </si>
+  <si>
+    <t>Sweden</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -352,14 +590,11 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -368,13 +603,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -705,9 +937,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDA0EEC7-A8A6-874F-BAA6-230636549D42}">
-  <dimension ref="A1:AJ4"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.95"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AJ19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.875" style="1" bestFit="1" customWidth="1"/>
@@ -715,8 +947,8 @@
     <col min="4" max="4" width="51.375" style="1" customWidth="1"/>
     <col min="5" max="6" width="47.125" style="1" customWidth="1"/>
     <col min="7" max="7" width="11.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.875" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.875" style="1" customWidth="1"/>
     <col min="11" max="11" width="18.375" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="24" style="1" bestFit="1" customWidth="1"/>
@@ -741,10 +973,11 @@
     <col min="34" max="34" width="10.625" style="1" customWidth="1"/>
     <col min="35" max="35" width="9.125" style="1" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="16384" width="10.875" style="1"/>
+    <col min="37" max="37" width="10.875" style="1" customWidth="1"/>
+    <col min="38" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="17.100000000000001">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -766,10 +999,10 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
@@ -854,233 +1087,768 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:36" ht="221.1">
+    <row r="2" spans="1:36" ht="408" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="1">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A3">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3">
+        <v>16.373799999999999</v>
+      </c>
+      <c r="I3">
+        <v>48.208199999999998</v>
+      </c>
+      <c r="J3" t="s">
+        <v>56</v>
+      </c>
+      <c r="R3" t="s">
+        <v>57</v>
+      </c>
+      <c r="S3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A4">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" t="s">
+        <v>64</v>
+      </c>
+      <c r="H4">
+        <v>13.404999999999999</v>
+      </c>
+      <c r="I4">
+        <v>52.52</v>
+      </c>
+      <c r="J4" t="s">
+        <v>65</v>
+      </c>
+      <c r="R4" t="s">
+        <v>66</v>
+      </c>
+      <c r="S4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A5">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H5">
+        <v>8.5417000000000005</v>
+      </c>
+      <c r="I5">
+        <v>47.376899999999999</v>
+      </c>
+      <c r="J5" t="s">
+        <v>74</v>
+      </c>
+      <c r="R5" t="s">
+        <v>75</v>
+      </c>
+      <c r="S5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>78</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A6">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6">
+        <v>2.3521999999999998</v>
+      </c>
+      <c r="I6">
+        <v>48.8566</v>
+      </c>
+      <c r="J6" t="s">
+        <v>82</v>
+      </c>
+      <c r="R6" t="s">
+        <v>83</v>
+      </c>
+      <c r="S6" t="s">
+        <v>84</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>85</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>87</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A7">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7">
+        <v>4.9040999999999997</v>
+      </c>
+      <c r="I7">
+        <v>52.367600000000003</v>
+      </c>
+      <c r="J7" t="s">
+        <v>91</v>
+      </c>
+      <c r="R7" t="s">
+        <v>92</v>
+      </c>
+      <c r="S7" t="s">
+        <v>93</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A8">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G8" t="s">
+        <v>97</v>
+      </c>
+      <c r="H8">
+        <v>4.3517000000000001</v>
+      </c>
+      <c r="I8">
+        <v>50.850299999999997</v>
+      </c>
+      <c r="J8" t="s">
+        <v>98</v>
+      </c>
+      <c r="R8" t="s">
+        <v>99</v>
+      </c>
+      <c r="S8" t="s">
+        <v>100</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>101</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>78</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H9">
+        <v>12.4964</v>
+      </c>
+      <c r="I9">
+        <v>41.902799999999999</v>
+      </c>
+      <c r="J9" t="s">
+        <v>106</v>
+      </c>
+      <c r="R9" t="s">
+        <v>107</v>
+      </c>
+      <c r="S9" t="s">
+        <v>108</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>109</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A10">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" t="s">
+        <v>111</v>
+      </c>
+      <c r="G10" t="s">
+        <v>112</v>
+      </c>
+      <c r="H10">
+        <v>14.437799999999999</v>
+      </c>
+      <c r="I10">
+        <v>50.075499999999998</v>
+      </c>
+      <c r="J10" t="s">
+        <v>113</v>
+      </c>
+      <c r="R10" t="s">
+        <v>114</v>
+      </c>
+      <c r="S10" t="s">
+        <v>115</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A11">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" t="s">
+        <v>118</v>
+      </c>
+      <c r="G11" t="s">
+        <v>119</v>
+      </c>
+      <c r="H11">
+        <v>21.0122</v>
+      </c>
+      <c r="I11">
+        <v>52.229700000000001</v>
+      </c>
+      <c r="J11" t="s">
+        <v>120</v>
+      </c>
+      <c r="R11" t="s">
+        <v>121</v>
+      </c>
+      <c r="S11" t="s">
+        <v>122</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>87</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A12">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" t="s">
+        <v>125</v>
+      </c>
+      <c r="G12" t="s">
+        <v>126</v>
+      </c>
+      <c r="H12">
+        <v>11.582000000000001</v>
+      </c>
+      <c r="I12">
+        <v>48.135100000000001</v>
+      </c>
+      <c r="J12" t="s">
+        <v>127</v>
+      </c>
+      <c r="R12" t="s">
+        <v>128</v>
+      </c>
+      <c r="S12" t="s">
+        <v>129</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A13">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" t="s">
+        <v>131</v>
+      </c>
+      <c r="G13" t="s">
+        <v>132</v>
+      </c>
+      <c r="H13">
+        <v>17.107700000000001</v>
+      </c>
+      <c r="I13">
+        <v>48.148600000000002</v>
+      </c>
+      <c r="J13" t="s">
+        <v>133</v>
+      </c>
+      <c r="R13" t="s">
+        <v>134</v>
+      </c>
+      <c r="S13" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>136</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A14">
+        <v>15</v>
+      </c>
+      <c r="B14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C14" t="s">
+        <v>138</v>
+      </c>
+      <c r="G14" t="s">
+        <v>139</v>
+      </c>
+      <c r="H14">
+        <v>14.505800000000001</v>
+      </c>
+      <c r="I14">
+        <v>46.056899999999999</v>
+      </c>
+      <c r="J14" t="s">
+        <v>140</v>
+      </c>
+      <c r="R14" t="s">
+        <v>141</v>
+      </c>
+      <c r="S14" t="s">
+        <v>142</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>143</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>87</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A15">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C15" t="s">
+        <v>145</v>
+      </c>
+      <c r="G15" t="s">
+        <v>146</v>
+      </c>
+      <c r="H15">
+        <v>11.4041</v>
+      </c>
+      <c r="I15">
+        <v>47.269199999999998</v>
+      </c>
+      <c r="J15" t="s">
+        <v>147</v>
+      </c>
+      <c r="R15" t="s">
+        <v>148</v>
+      </c>
+      <c r="S15" t="s">
+        <v>149</v>
+      </c>
+      <c r="AD15" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE2" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AF2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AG2" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH2" s="1" t="s">
-        <v>56</v>
+      <c r="AE15" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:36" ht="119.1">
-      <c r="A3" s="1">
-        <v>6</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" s="1" t="s">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.5">
+      <c r="A16">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C16" t="s">
+        <v>151</v>
+      </c>
+      <c r="G16" t="s">
+        <v>152</v>
+      </c>
+      <c r="H16">
+        <v>7.4474</v>
+      </c>
+      <c r="I16">
+        <v>46.948</v>
+      </c>
+      <c r="J16" t="s">
+        <v>153</v>
+      </c>
+      <c r="R16" t="s">
+        <v>154</v>
+      </c>
+      <c r="S16" t="s">
+        <v>155</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>77</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>78</v>
+      </c>
+      <c r="AF16" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="AG16" t="s">
         <v>61</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q3" s="1" t="s">
+    </row>
+    <row r="17" spans="1:33" x14ac:dyDescent="0.5">
+      <c r="A17">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>156</v>
+      </c>
+      <c r="C17" t="s">
+        <v>157</v>
+      </c>
+      <c r="G17" t="s">
+        <v>158</v>
+      </c>
+      <c r="H17">
+        <v>4.8357000000000001</v>
+      </c>
+      <c r="I17">
+        <v>45.764000000000003</v>
+      </c>
+      <c r="J17" t="s">
+        <v>159</v>
+      </c>
+      <c r="R17" t="s">
+        <v>160</v>
+      </c>
+      <c r="S17" t="s">
+        <v>161</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>85</v>
+      </c>
+      <c r="AE17" t="s">
         <v>69</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="AF17" t="s">
         <v>70</v>
       </c>
-      <c r="S3" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="U3" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="AD3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE3" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AF3" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="AG3" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH3" s="1" t="s">
-        <v>56</v>
+      <c r="AG17" t="s">
+        <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:36" ht="408" customHeight="1">
-      <c r="A4" s="1">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.5">
+      <c r="A18">
         <v>19</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B18" t="s">
+        <v>162</v>
+      </c>
+      <c r="C18" t="s">
+        <v>163</v>
+      </c>
+      <c r="G18" t="s">
+        <v>164</v>
+      </c>
+      <c r="H18">
+        <v>12.568300000000001</v>
+      </c>
+      <c r="I18">
+        <v>55.676099999999998</v>
+      </c>
+      <c r="J18" t="s">
+        <v>165</v>
+      </c>
+      <c r="R18" t="s">
+        <v>166</v>
+      </c>
+      <c r="S18" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>168</v>
+      </c>
+      <c r="AE18" t="s">
         <v>78</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="O4" s="1" t="s">
+      <c r="AF18" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:33" x14ac:dyDescent="0.5">
+      <c r="A19">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
+        <v>169</v>
+      </c>
+      <c r="C19" t="s">
+        <v>170</v>
+      </c>
+      <c r="G19" t="s">
+        <v>171</v>
+      </c>
+      <c r="H19">
+        <v>18.0686</v>
+      </c>
+      <c r="I19">
+        <v>59.329300000000003</v>
+      </c>
+      <c r="J19" t="s">
+        <v>172</v>
+      </c>
+      <c r="R19" t="s">
+        <v>173</v>
+      </c>
+      <c r="S19" t="s">
+        <v>174</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>175</v>
+      </c>
+      <c r="AE19" t="s">
         <v>86</v>
       </c>
-      <c r="P4" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="U4" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="AF4" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="AH4" s="1" t="s">
-        <v>56</v>
+      <c r="AF19" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG19" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="S2" r:id="rId1" xr:uid="{194014FF-AC62-4B4B-A40F-E47E8D41346E}"/>
-    <hyperlink ref="U2" r:id="rId2" xr:uid="{D6384DAB-A00C-A041-B970-C8B0B1CC6902}"/>
-    <hyperlink ref="J2" r:id="rId3" xr:uid="{7F4D688E-667A-6F4B-8144-2D765F3B24E8}"/>
-    <hyperlink ref="J3" r:id="rId4" xr:uid="{13345165-5C3B-094A-A57A-D3D940031F08}"/>
-    <hyperlink ref="S3" r:id="rId5" xr:uid="{E8266283-AADF-3444-AFBA-F8A4A9FA03D2}"/>
-    <hyperlink ref="U3" r:id="rId6" xr:uid="{95A75298-1840-3D48-878B-D2F4D6F26002}"/>
-    <hyperlink ref="U4" r:id="rId7" xr:uid="{AEBA8EB5-96B7-504F-8727-B48413D3685A}"/>
+    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>